<commit_message>
Sprint 2b: Fix national notice compatibility in classifier + exporter
- classifier.py: _build_prompt() and _haiku_prefilter() now fall back to
  _title_final / _national_raw_text / _authority_name for DE-SB and PL-BZP
  notices that don't carry standard TED title/description fields
- exporter.py: _flatten_notice() adds national-format fallbacks for
  authority name, country, publication date (_pub_date_clean), value
  (_value_amount/_value_currency), winner, and description
- Add src/de_scraper.py and src/pl_scraper.py (legacy scraper modules)
- Export updated: 260427_TED_Tender Data_00.01.xlsx (143 rows, 23 cols)

Note: 564 national notices (115 DE-SB + 449 PL-BZP) were correctly
rejected by Haiku pre-filter — all civilian procurement, no military
trailer notices in the current national scraper results. PL adapter
needs CPV+wojsk combined search to fetch actual military trailer notices.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Vorlage.xlsx
+++ b/Vorlage.xlsx
@@ -107,7 +107,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -148,6 +148,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="001F4E79"/>
         <bgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00548235"/>
+        <bgColor rgb="00548235"/>
       </patternFill>
     </fill>
   </fills>
@@ -213,7 +219,7 @@
     <xf numFmtId="49" fontId="7" fillId="0" borderId="4"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="4"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -249,6 +255,9 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2509,6 +2518,8 @@
     <col width="30" customWidth="1" min="16" max="16"/>
     <col width="45" customWidth="1" min="17" max="17"/>
     <col width="65" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="23" max="23"/>
+    <col width="45" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2686,10 +2697,22 @@
         </is>
       </c>
       <c r="T4" s="19" t="n"/>
-      <c r="U4" s="19" t="n"/>
+      <c r="U4" s="19" t="inlineStr">
+        <is>
+          <t>Source URL (TED)</t>
+        </is>
+      </c>
       <c r="V4" s="19" t="n"/>
-      <c r="W4" s="19" t="n"/>
-      <c r="X4" s="19" t="n"/>
+      <c r="W4" s="23" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="X4" s="23" t="inlineStr">
+        <is>
+          <t>Source URL (National)</t>
+        </is>
+      </c>
       <c r="Y4" s="19" t="n"/>
     </row>
     <row r="5">

</xml_diff>